<commit_message>
* billing settings added to runtime_setting * Added description field to runtime_setting
</commit_message>
<xml_diff>
--- a/docs/SFTPManager-Test-Plan.xlsx
+++ b/docs/SFTPManager-Test-Plan.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\joema\OneDrive\Documents\NetBeansProjects\SFTPManager\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\joema\Downloads\sftp-manager\sftp-manager\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8A3C61EE-F537-4431-ACAE-0B8FF69E35EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18D87BE3-8117-47E1-B9AE-00657FA00DE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="816" yWindow="756" windowWidth="14148" windowHeight="9492" xr2:uid="{3AB46E1C-6979-4AE0-A30D-F087EBE6ECB8}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="27885" windowHeight="16440" firstSheet="5" activeTab="7" xr2:uid="{3AB46E1C-6979-4AE0-A30D-F087EBE6ECB8}"/>
   </bookViews>
   <sheets>
     <sheet name="Index" sheetId="1" r:id="rId1"/>
@@ -71,7 +71,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1565" uniqueCount="1058">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1688" uniqueCount="1094">
   <si>
     <t>ID</t>
   </si>
@@ -3245,13 +3245,121 @@
   </si>
   <si>
     <t>TOTAL</t>
+  </si>
+  <si>
+    <t>Outcome</t>
+  </si>
+  <si>
+    <t>SUCCESS</t>
+  </si>
+  <si>
+    <t>Issues</t>
+  </si>
+  <si>
+    <t>When I create TWO SFTP Services, they can't have IDENTICAL SFTP logins Service Accounts, e.g. joe for both of them.</t>
+  </si>
+  <si>
+    <t>???</t>
+  </si>
+  <si>
+    <t>Not sure how to do.</t>
+  </si>
+  <si>
+    <t>When I go to delete a USER from the ADMIN interface, it doesn’t delete the user!</t>
+  </si>
+  <si>
+    <t>SEMI-SUCCESS</t>
+  </si>
+  <si>
+    <t>User can reset password themselves…. And this also unlocks the account</t>
+  </si>
+  <si>
+    <t>FAILED</t>
+  </si>
+  <si>
+    <t>It recognises that this account hasn't been created and prompts for creation of new account.</t>
+  </si>
+  <si>
+    <t>IT returns 401 in console, but no message</t>
+  </si>
+  <si>
+    <t>FIXED</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>Remediation</t>
+  </si>
+  <si>
+    <t>Fixed!</t>
+  </si>
+  <si>
+    <t>Dates are in American format - not good.</t>
+  </si>
+  <si>
+    <t>NOT TESTED YET</t>
+  </si>
+  <si>
+    <t>Popup appears!</t>
+  </si>
+  <si>
+    <t>Can put extra long mobile # in . Can put in dodgy long postcode</t>
+  </si>
+  <si>
+    <t>IT just sets it… and no paymenet because no card has been added.</t>
+  </si>
+  <si>
+    <t>no idea why test case mentions PATCH</t>
+  </si>
+  <si>
+    <t>But when I try to re-create account, there are some entries somewhere that need to be deleted…</t>
+  </si>
+  <si>
+    <t>Deleted email_notifications entries and payments entries AND it archives payment information</t>
+  </si>
+  <si>
+    <t>IF a PORTAL user tries to add additional SFTP Services, it doesn't allow one to</t>
+  </si>
+  <si>
+    <t>But noticed the DELETION from portal doesn't work!</t>
+  </si>
+  <si>
+    <t>We have no plans with unlimited space. So we ignore this.</t>
+  </si>
+  <si>
+    <t>Session still active</t>
+  </si>
+  <si>
+    <t>Fixed issue in PORTAL</t>
+  </si>
+  <si>
+    <t>Ran /api/users and didn't see password at all</t>
+  </si>
+  <si>
+    <t>IT is shown</t>
+  </si>
+  <si>
+    <t>SKIP</t>
+  </si>
+  <si>
+    <t>We allow usernames to be duplicated. The Login is what ths unique and combines the username entered and the SFTP Service short name</t>
+  </si>
+  <si>
+    <t>WE NEED TO Make it do backend checks!!</t>
+  </si>
+  <si>
+    <t>deleting the Serivce Account</t>
+  </si>
+  <si>
+    <t>2026-07-31 07:10:01,067 mod_wrap2/2.0.7[436052]: warning: bad net/mask expression: '172.105.168.0/24'. Individual IPS work</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -3300,8 +3408,22 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="12">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -3338,8 +3460,38 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -3362,11 +3514,32 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFC8C8C8"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFC8C8C8"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFC8C8C8"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -3392,16 +3565,53 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -3734,243 +3944,254 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6CD14F39-B8EC-4EBF-BF0C-64C380DA09A2}">
-  <dimension ref="A1:B30"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:B37"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="95.77734375" customWidth="1"/>
-    <col min="2" max="2" width="14.77734375" customWidth="1"/>
+    <col min="1" max="1" width="95.7109375" customWidth="1"/>
+    <col min="2" max="2" width="14.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="23.4" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:2" ht="24" x14ac:dyDescent="0.4">
       <c r="A1" s="9" t="s">
         <v>1029</v>
       </c>
-      <c r="B1" s="10"/>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A2" s="11" t="s">
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="10" t="s">
         <v>1030</v>
       </c>
-      <c r="B2" s="10"/>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A3" s="12" t="s">
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" s="11" t="s">
         <v>1031</v>
       </c>
-      <c r="B3" s="10"/>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A4" s="10"/>
-      <c r="B4" s="10"/>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A5" s="13" t="s">
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="12" t="s">
         <v>1032</v>
       </c>
-      <c r="B5" s="10"/>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>1033</v>
       </c>
-      <c r="B6" s="10"/>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    </row>
+    <row r="7" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>1034</v>
       </c>
-      <c r="B7" s="10"/>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+    </row>
+    <row r="8" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>1035</v>
       </c>
-      <c r="B8" s="10"/>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+    </row>
+    <row r="9" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>1036</v>
       </c>
-      <c r="B9" s="10"/>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>1037</v>
       </c>
-      <c r="B10" s="10"/>
-    </row>
-    <row r="11" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+    </row>
+    <row r="11" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>1038</v>
       </c>
-      <c r="B11" s="10"/>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+    </row>
+    <row r="12" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>1039</v>
       </c>
-      <c r="B12" s="10"/>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A13" s="10"/>
-      <c r="B13" s="10"/>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A14" s="14" t="s">
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" s="13" t="s">
         <v>1040</v>
       </c>
-      <c r="B14" s="14" t="s">
+      <c r="B14" s="13" t="s">
         <v>1041</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A15" s="15" t="s">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" s="14" t="s">
         <v>1042</v>
       </c>
-      <c r="B15" s="15">
+      <c r="B15" s="14">
         <v>20</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A16" s="15" t="s">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" s="14" t="s">
         <v>1043</v>
       </c>
-      <c r="B16" s="15">
+      <c r="B16" s="14">
         <v>10</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A17" s="15" t="s">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" s="14" t="s">
         <v>1044</v>
       </c>
-      <c r="B17" s="15">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" s="15" t="s">
+      <c r="B17" s="14">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" s="14" t="s">
         <v>1045</v>
       </c>
-      <c r="B18" s="15">
+      <c r="B18" s="14">
         <v>8</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A19" s="15" t="s">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" s="14" t="s">
         <v>1046</v>
       </c>
-      <c r="B19" s="15">
+      <c r="B19" s="14">
         <v>12</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A20" s="15" t="s">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" s="14" t="s">
         <v>1047</v>
       </c>
-      <c r="B20" s="15">
+      <c r="B20" s="14">
         <v>8</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A21" s="15" t="s">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" s="14" t="s">
         <v>1048</v>
       </c>
-      <c r="B21" s="15">
+      <c r="B21" s="14">
         <v>8</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A22" s="15" t="s">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" s="14" t="s">
         <v>1049</v>
       </c>
-      <c r="B22" s="15">
+      <c r="B22" s="14">
         <v>6</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A23" s="15" t="s">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" s="14" t="s">
         <v>1050</v>
       </c>
-      <c r="B23" s="15">
+      <c r="B23" s="14">
         <v>15</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A24" s="15" t="s">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" s="14" t="s">
         <v>1051</v>
       </c>
-      <c r="B24" s="15">
+      <c r="B24" s="14">
         <v>16</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A25" s="15" t="s">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" s="14" t="s">
         <v>1052</v>
       </c>
-      <c r="B25" s="15">
+      <c r="B25" s="14">
         <v>10</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A26" s="15" t="s">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26" s="14" t="s">
         <v>1053</v>
       </c>
-      <c r="B26" s="15">
+      <c r="B26" s="14">
         <v>8</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A27" s="15" t="s">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A27" s="14" t="s">
         <v>1054</v>
       </c>
-      <c r="B27" s="15">
+      <c r="B27" s="14">
         <v>16</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A28" s="15" t="s">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A28" s="14" t="s">
         <v>1055</v>
       </c>
-      <c r="B28" s="15">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A29" s="15" t="s">
+      <c r="B28" s="14">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A29" s="14" t="s">
         <v>1056</v>
       </c>
-      <c r="B29" s="15">
+      <c r="B29" s="14">
         <v>12</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A30" s="16" t="s">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A30" s="15" t="s">
         <v>1057</v>
       </c>
-      <c r="B30" s="16">
+      <c r="B30" s="15">
         <v>177</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A34" s="11" t="s">
+        <v>1060</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>1061</v>
+      </c>
+      <c r="B35" s="23" t="s">
+        <v>1073</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>1064</v>
+      </c>
+      <c r="B36" s="23" t="s">
+        <v>1073</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>1074</v>
+      </c>
+      <c r="B37" s="23" t="s">
+        <v>1073</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE4B2888-C380-42AB-B6FF-7902ECD4725D}">
   <dimension ref="A1:H16"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.77734375" customWidth="1"/>
-    <col min="2" max="3" width="34.77734375" customWidth="1"/>
-    <col min="4" max="4" width="42.77734375" customWidth="1"/>
-    <col min="5" max="5" width="26.77734375" customWidth="1"/>
-    <col min="6" max="6" width="42.77734375" customWidth="1"/>
-    <col min="7" max="7" width="10.77734375" customWidth="1"/>
-    <col min="8" max="8" width="12.77734375" customWidth="1"/>
+    <col min="1" max="1" width="12.7109375" customWidth="1"/>
+    <col min="2" max="3" width="34.7109375" customWidth="1"/>
+    <col min="4" max="4" width="42.7109375" customWidth="1"/>
+    <col min="5" max="5" width="26.7109375" customWidth="1"/>
+    <col min="6" max="6" width="42.7109375" customWidth="1"/>
+    <col min="7" max="7" width="10.7109375" customWidth="1"/>
+    <col min="8" max="8" width="12.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -3996,7 +4217,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>509</v>
       </c>
@@ -4022,7 +4243,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>515</v>
       </c>
@@ -4048,7 +4269,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>521</v>
       </c>
@@ -4074,7 +4295,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
         <v>527</v>
       </c>
@@ -4100,7 +4321,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>532</v>
       </c>
@@ -4126,7 +4347,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
         <v>538</v>
       </c>
@@ -4152,7 +4373,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>544</v>
       </c>
@@ -4178,7 +4399,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
         <v>550</v>
       </c>
@@ -4204,7 +4425,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>555</v>
       </c>
@@ -4230,7 +4451,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
         <v>560</v>
       </c>
@@ -4256,7 +4477,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>566</v>
       </c>
@@ -4282,7 +4503,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
         <v>572</v>
       </c>
@@ -4308,7 +4529,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>578</v>
       </c>
@@ -4334,7 +4555,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
         <v>583</v>
       </c>
@@ -4360,7 +4581,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>589</v>
       </c>
@@ -4395,18 +4616,18 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B2D9B15-1B7B-4FEB-A8CA-6B9AA2105BC3}">
   <dimension ref="A1:H17"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.77734375" customWidth="1"/>
-    <col min="2" max="3" width="34.77734375" customWidth="1"/>
-    <col min="4" max="4" width="42.77734375" customWidth="1"/>
-    <col min="5" max="5" width="26.77734375" customWidth="1"/>
-    <col min="6" max="6" width="42.77734375" customWidth="1"/>
-    <col min="7" max="7" width="10.77734375" customWidth="1"/>
-    <col min="8" max="8" width="12.77734375" customWidth="1"/>
+    <col min="1" max="1" width="12.7109375" customWidth="1"/>
+    <col min="2" max="3" width="34.7109375" customWidth="1"/>
+    <col min="4" max="4" width="42.7109375" customWidth="1"/>
+    <col min="5" max="5" width="26.7109375" customWidth="1"/>
+    <col min="6" max="6" width="42.7109375" customWidth="1"/>
+    <col min="7" max="7" width="10.7109375" customWidth="1"/>
+    <col min="8" max="8" width="12.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -4432,7 +4653,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>594</v>
       </c>
@@ -4458,7 +4679,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>600</v>
       </c>
@@ -4484,7 +4705,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>606</v>
       </c>
@@ -4510,7 +4731,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
         <v>612</v>
       </c>
@@ -4536,7 +4757,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>618</v>
       </c>
@@ -4562,7 +4783,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
         <v>624</v>
       </c>
@@ -4588,7 +4809,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>630</v>
       </c>
@@ -4614,7 +4835,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
         <v>636</v>
       </c>
@@ -4640,7 +4861,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>642</v>
       </c>
@@ -4666,7 +4887,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
         <v>647</v>
       </c>
@@ -4692,7 +4913,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>653</v>
       </c>
@@ -4718,7 +4939,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
         <v>659</v>
       </c>
@@ -4744,7 +4965,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>665</v>
       </c>
@@ -4770,7 +4991,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
         <v>671</v>
       </c>
@@ -4796,7 +5017,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>676</v>
       </c>
@@ -4822,7 +5043,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
         <v>682</v>
       </c>
@@ -4857,18 +5078,18 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{490693A7-B281-4E98-B0D4-3E2612AF40D7}">
   <dimension ref="A1:H11"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.77734375" customWidth="1"/>
-    <col min="2" max="3" width="34.77734375" customWidth="1"/>
-    <col min="4" max="4" width="42.77734375" customWidth="1"/>
-    <col min="5" max="5" width="26.77734375" customWidth="1"/>
-    <col min="6" max="6" width="42.77734375" customWidth="1"/>
-    <col min="7" max="7" width="10.77734375" customWidth="1"/>
-    <col min="8" max="8" width="12.77734375" customWidth="1"/>
+    <col min="1" max="1" width="12.7109375" customWidth="1"/>
+    <col min="2" max="3" width="34.7109375" customWidth="1"/>
+    <col min="4" max="4" width="42.7109375" customWidth="1"/>
+    <col min="5" max="5" width="26.7109375" customWidth="1"/>
+    <col min="6" max="6" width="42.7109375" customWidth="1"/>
+    <col min="7" max="7" width="10.7109375" customWidth="1"/>
+    <col min="8" max="8" width="12.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -4894,7 +5115,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>688</v>
       </c>
@@ -4920,7 +5141,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>694</v>
       </c>
@@ -4946,7 +5167,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>699</v>
       </c>
@@ -4972,7 +5193,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
         <v>705</v>
       </c>
@@ -4998,7 +5219,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>711</v>
       </c>
@@ -5024,7 +5245,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
         <v>717</v>
       </c>
@@ -5050,7 +5271,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>722</v>
       </c>
@@ -5076,7 +5297,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
         <v>727</v>
       </c>
@@ -5102,7 +5323,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>733</v>
       </c>
@@ -5128,7 +5349,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
         <v>739</v>
       </c>
@@ -5163,18 +5384,18 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{10F29A35-B863-4444-917C-00415C8184F1}">
   <dimension ref="A1:H9"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.77734375" customWidth="1"/>
-    <col min="2" max="3" width="34.77734375" customWidth="1"/>
-    <col min="4" max="4" width="42.77734375" customWidth="1"/>
-    <col min="5" max="5" width="26.77734375" customWidth="1"/>
-    <col min="6" max="6" width="42.77734375" customWidth="1"/>
-    <col min="7" max="7" width="10.77734375" customWidth="1"/>
-    <col min="8" max="8" width="12.77734375" customWidth="1"/>
+    <col min="1" max="1" width="12.7109375" customWidth="1"/>
+    <col min="2" max="3" width="34.7109375" customWidth="1"/>
+    <col min="4" max="4" width="42.7109375" customWidth="1"/>
+    <col min="5" max="5" width="26.7109375" customWidth="1"/>
+    <col min="6" max="6" width="42.7109375" customWidth="1"/>
+    <col min="7" max="7" width="10.7109375" customWidth="1"/>
+    <col min="8" max="8" width="12.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -5200,7 +5421,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>745</v>
       </c>
@@ -5226,7 +5447,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>750</v>
       </c>
@@ -5252,7 +5473,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>755</v>
       </c>
@@ -5278,7 +5499,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
         <v>760</v>
       </c>
@@ -5304,7 +5525,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>766</v>
       </c>
@@ -5330,7 +5551,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
         <v>770</v>
       </c>
@@ -5356,7 +5577,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>776</v>
       </c>
@@ -5382,7 +5603,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
         <v>782</v>
       </c>
@@ -5417,18 +5638,18 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{30872A71-BC0A-46C8-ABE9-7B7574FF19B6}">
   <dimension ref="A1:H17"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.77734375" customWidth="1"/>
-    <col min="2" max="3" width="34.77734375" customWidth="1"/>
-    <col min="4" max="4" width="42.77734375" customWidth="1"/>
-    <col min="5" max="5" width="26.77734375" customWidth="1"/>
-    <col min="6" max="6" width="42.77734375" customWidth="1"/>
-    <col min="7" max="7" width="10.77734375" customWidth="1"/>
-    <col min="8" max="8" width="12.77734375" customWidth="1"/>
+    <col min="1" max="1" width="12.7109375" customWidth="1"/>
+    <col min="2" max="3" width="34.7109375" customWidth="1"/>
+    <col min="4" max="4" width="42.7109375" customWidth="1"/>
+    <col min="5" max="5" width="26.7109375" customWidth="1"/>
+    <col min="6" max="6" width="42.7109375" customWidth="1"/>
+    <col min="7" max="7" width="10.7109375" customWidth="1"/>
+    <col min="8" max="8" width="12.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -5454,7 +5675,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>788</v>
       </c>
@@ -5480,7 +5701,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>794</v>
       </c>
@@ -5506,7 +5727,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>800</v>
       </c>
@@ -5532,7 +5753,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
         <v>805</v>
       </c>
@@ -5558,7 +5779,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>811</v>
       </c>
@@ -5584,7 +5805,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
         <v>815</v>
       </c>
@@ -5610,7 +5831,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>821</v>
       </c>
@@ -5636,7 +5857,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
         <v>825</v>
       </c>
@@ -5662,7 +5883,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>830</v>
       </c>
@@ -5688,7 +5909,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
         <v>834</v>
       </c>
@@ -5714,7 +5935,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>840</v>
       </c>
@@ -5740,7 +5961,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
         <v>846</v>
       </c>
@@ -5766,7 +5987,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>852</v>
       </c>
@@ -5792,7 +6013,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
         <v>858</v>
       </c>
@@ -5818,7 +6039,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>864</v>
       </c>
@@ -5844,7 +6065,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
         <v>870</v>
       </c>
@@ -5879,18 +6100,18 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7349428E-5EA3-479F-896A-8429486CF7D4}">
   <dimension ref="A1:H15"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.77734375" customWidth="1"/>
-    <col min="2" max="3" width="34.77734375" customWidth="1"/>
-    <col min="4" max="4" width="42.77734375" customWidth="1"/>
-    <col min="5" max="5" width="26.77734375" customWidth="1"/>
-    <col min="6" max="6" width="42.77734375" customWidth="1"/>
-    <col min="7" max="7" width="10.77734375" customWidth="1"/>
-    <col min="8" max="8" width="12.77734375" customWidth="1"/>
+    <col min="1" max="1" width="12.7109375" customWidth="1"/>
+    <col min="2" max="3" width="34.7109375" customWidth="1"/>
+    <col min="4" max="4" width="42.7109375" customWidth="1"/>
+    <col min="5" max="5" width="26.7109375" customWidth="1"/>
+    <col min="6" max="6" width="42.7109375" customWidth="1"/>
+    <col min="7" max="7" width="10.7109375" customWidth="1"/>
+    <col min="8" max="8" width="12.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -5916,7 +6137,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>875</v>
       </c>
@@ -5942,7 +6163,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>881</v>
       </c>
@@ -5968,7 +6189,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>887</v>
       </c>
@@ -5994,7 +6215,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
         <v>893</v>
       </c>
@@ -6020,7 +6241,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>899</v>
       </c>
@@ -6046,7 +6267,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
         <v>905</v>
       </c>
@@ -6072,7 +6293,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>911</v>
       </c>
@@ -6098,7 +6319,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
         <v>917</v>
       </c>
@@ -6124,7 +6345,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>922</v>
       </c>
@@ -6150,7 +6371,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
         <v>928</v>
       </c>
@@ -6176,7 +6397,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>934</v>
       </c>
@@ -6202,7 +6423,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
         <v>940</v>
       </c>
@@ -6228,7 +6449,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>946</v>
       </c>
@@ -6254,7 +6475,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
         <v>952</v>
       </c>
@@ -6289,18 +6510,18 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{84A759D0-43E7-4F51-9AA6-5FDF91604FF2}">
   <dimension ref="A1:H13"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.77734375" customWidth="1"/>
-    <col min="2" max="3" width="34.77734375" customWidth="1"/>
-    <col min="4" max="4" width="42.77734375" customWidth="1"/>
-    <col min="5" max="5" width="26.77734375" customWidth="1"/>
-    <col min="6" max="6" width="42.77734375" customWidth="1"/>
-    <col min="7" max="7" width="10.77734375" customWidth="1"/>
-    <col min="8" max="8" width="12.77734375" customWidth="1"/>
+    <col min="1" max="1" width="12.7109375" customWidth="1"/>
+    <col min="2" max="3" width="34.7109375" customWidth="1"/>
+    <col min="4" max="4" width="42.7109375" customWidth="1"/>
+    <col min="5" max="5" width="26.7109375" customWidth="1"/>
+    <col min="6" max="6" width="42.7109375" customWidth="1"/>
+    <col min="7" max="7" width="10.7109375" customWidth="1"/>
+    <col min="8" max="8" width="12.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -6326,7 +6547,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>958</v>
       </c>
@@ -6352,7 +6573,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>964</v>
       </c>
@@ -6378,7 +6599,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>970</v>
       </c>
@@ -6404,7 +6625,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="72" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" ht="90" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
         <v>976</v>
       </c>
@@ -6430,7 +6651,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>982</v>
       </c>
@@ -6456,7 +6677,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
         <v>988</v>
       </c>
@@ -6482,7 +6703,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>994</v>
       </c>
@@ -6508,7 +6729,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
         <v>1000</v>
       </c>
@@ -6534,7 +6755,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>1006</v>
       </c>
@@ -6560,7 +6781,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
         <v>1011</v>
       </c>
@@ -6586,7 +6807,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>1017</v>
       </c>
@@ -6612,7 +6833,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" ht="75" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
         <v>1023</v>
       </c>
@@ -6646,19 +6867,21 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{366D77D7-C10E-42A0-950B-F3568D7ED79B}">
-  <dimension ref="A1:H21"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:K21"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.77734375" customWidth="1"/>
-    <col min="2" max="3" width="34.77734375" customWidth="1"/>
-    <col min="4" max="4" width="42.77734375" customWidth="1"/>
-    <col min="5" max="5" width="26.77734375" customWidth="1"/>
-    <col min="6" max="6" width="42.77734375" customWidth="1"/>
-    <col min="7" max="7" width="10.77734375" customWidth="1"/>
-    <col min="8" max="8" width="12.77734375" customWidth="1"/>
+    <col min="1" max="1" width="12.7109375" customWidth="1"/>
+    <col min="2" max="3" width="34.7109375" customWidth="1"/>
+    <col min="4" max="4" width="42.7109375" customWidth="1"/>
+    <col min="5" max="5" width="26.7109375" customWidth="1"/>
+    <col min="6" max="6" width="42.7109375" customWidth="1"/>
+    <col min="7" max="7" width="10.7109375" customWidth="1"/>
+    <col min="8" max="8" width="12.7109375" customWidth="1"/>
+    <col min="10" max="10" width="16.7109375" customWidth="1"/>
+    <col min="11" max="11" width="12.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -6683,8 +6906,17 @@
       <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="I1" s="16" t="s">
+        <v>1058</v>
+      </c>
+      <c r="J1" s="16" t="s">
+        <v>1071</v>
+      </c>
+      <c r="K1" s="16" t="s">
+        <v>1072</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>8</v>
       </c>
@@ -6709,8 +6941,11 @@
       <c r="H2" s="3" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="I2" s="25" t="s">
+        <v>1059</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>16</v>
       </c>
@@ -6735,8 +6970,11 @@
       <c r="H3" s="5" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="I3" s="25" t="s">
+        <v>1059</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>23</v>
       </c>
@@ -6761,8 +6999,11 @@
       <c r="H4" s="3" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="I4" s="25" t="s">
+        <v>1059</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
         <v>29</v>
       </c>
@@ -6775,7 +7016,7 @@
       <c r="D5" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="E5" s="19" t="s">
         <v>33</v>
       </c>
       <c r="F5" s="5" t="s">
@@ -6787,8 +7028,11 @@
       <c r="H5" s="5" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="6" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="I5" s="25" t="s">
+        <v>1059</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>35</v>
       </c>
@@ -6813,8 +7057,11 @@
       <c r="H6" s="3" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="7" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="I6" s="25" t="s">
+        <v>1059</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
         <v>43</v>
       </c>
@@ -6839,8 +7086,14 @@
       <c r="H7" s="5" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="8" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="I7" s="24" t="s">
+        <v>1062</v>
+      </c>
+      <c r="J7" s="18" t="s">
+        <v>1063</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>48</v>
       </c>
@@ -6865,8 +7118,11 @@
       <c r="H8" s="3" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="9" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="I8" s="25" t="s">
+        <v>1059</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
         <v>54</v>
       </c>
@@ -6891,8 +7147,11 @@
       <c r="H9" s="5" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="10" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="I9" s="25" t="s">
+        <v>1059</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" ht="90" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>60</v>
       </c>
@@ -6917,8 +7176,14 @@
       <c r="H10" s="3" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="11" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="I10" s="25" t="s">
+        <v>1065</v>
+      </c>
+      <c r="J10" s="17" t="s">
+        <v>1066</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
         <v>66</v>
       </c>
@@ -6943,8 +7208,11 @@
       <c r="H11" s="5" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="12" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="I11" s="25" t="s">
+        <v>1059</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>72</v>
       </c>
@@ -6969,8 +7237,11 @@
       <c r="H12" s="3" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="13" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="I12" s="25" t="s">
+        <v>1059</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
         <v>78</v>
       </c>
@@ -6995,8 +7266,11 @@
       <c r="H13" s="5" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="14" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="I13" s="25" t="s">
+        <v>1059</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>84</v>
       </c>
@@ -7021,8 +7295,11 @@
       <c r="H14" s="3" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="15" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="I14" s="25" t="s">
+        <v>1059</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
         <v>90</v>
       </c>
@@ -7047,8 +7324,11 @@
       <c r="H15" s="5" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="16" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="I15" s="25" t="s">
+        <v>1059</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>96</v>
       </c>
@@ -7061,7 +7341,7 @@
       <c r="D16" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="E16" s="3" t="s">
+      <c r="E16" s="20" t="s">
         <v>100</v>
       </c>
       <c r="F16" s="3" t="s">
@@ -7073,8 +7353,14 @@
       <c r="H16" s="3" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="17" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="I16" s="21" t="s">
+        <v>1067</v>
+      </c>
+      <c r="J16" t="s">
+        <v>1068</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
         <v>102</v>
       </c>
@@ -7099,8 +7385,11 @@
       <c r="H17" s="5" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="18" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="I17" s="25" t="s">
+        <v>1059</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
         <v>106</v>
       </c>
@@ -7125,8 +7414,11 @@
       <c r="H18" s="3" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="19" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="I18" s="25" t="s">
+        <v>1059</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
         <v>112</v>
       </c>
@@ -7151,8 +7443,11 @@
       <c r="H19" s="5" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="20" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="I19" s="25" t="s">
+        <v>1059</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
         <v>118</v>
       </c>
@@ -7177,8 +7472,17 @@
       <c r="H20" s="3" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="21" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="I20" s="21" t="s">
+        <v>1067</v>
+      </c>
+      <c r="J20" s="17" t="s">
+        <v>1069</v>
+      </c>
+      <c r="K20" s="22" t="s">
+        <v>1070</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
         <v>124</v>
       </c>
@@ -7203,28 +7507,35 @@
       <c r="H21" s="5" t="s">
         <v>131</v>
       </c>
+      <c r="I21" s="25" t="s">
+        <v>1059</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:H21" xr:uid="{366D77D7-C10E-42A0-950B-F3568D7ED79B}"/>
+  <hyperlinks>
+    <hyperlink ref="E5" r:id="rId1" xr:uid="{ACB8BED5-76C9-4735-AC48-E46B8B80638D}"/>
+    <hyperlink ref="E16" r:id="rId2" xr:uid="{463EAA50-37A6-48C4-9805-30F733B0948B}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D645DA2-14F1-4A95-BD2E-B7BB26CB17DA}">
-  <dimension ref="A1:H11"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:K11"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.77734375" customWidth="1"/>
-    <col min="2" max="3" width="34.77734375" customWidth="1"/>
-    <col min="4" max="4" width="42.77734375" customWidth="1"/>
-    <col min="5" max="5" width="26.77734375" customWidth="1"/>
-    <col min="6" max="6" width="42.77734375" customWidth="1"/>
-    <col min="7" max="7" width="10.77734375" customWidth="1"/>
-    <col min="8" max="8" width="12.77734375" customWidth="1"/>
+    <col min="1" max="1" width="12.7109375" customWidth="1"/>
+    <col min="2" max="3" width="34.7109375" customWidth="1"/>
+    <col min="4" max="4" width="42.7109375" customWidth="1"/>
+    <col min="5" max="5" width="26.7109375" customWidth="1"/>
+    <col min="6" max="6" width="42.7109375" customWidth="1"/>
+    <col min="7" max="7" width="10.7109375" customWidth="1"/>
+    <col min="8" max="8" width="12.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -7249,8 +7560,17 @@
       <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="I1" s="16" t="s">
+        <v>1058</v>
+      </c>
+      <c r="J1" s="16" t="s">
+        <v>1071</v>
+      </c>
+      <c r="K1" s="16" t="s">
+        <v>1072</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>132</v>
       </c>
@@ -7275,8 +7595,11 @@
       <c r="H2" s="3" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="I2" s="22" t="s">
+        <v>1059</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>138</v>
       </c>
@@ -7301,8 +7624,11 @@
       <c r="H3" s="5" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="I3" s="22" t="s">
+        <v>1059</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>144</v>
       </c>
@@ -7327,8 +7653,11 @@
       <c r="H4" s="3" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="I4" s="22" t="s">
+        <v>1059</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
         <v>149</v>
       </c>
@@ -7353,8 +7682,11 @@
       <c r="H5" s="5" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="6" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="I5" s="22" t="s">
+        <v>1059</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>155</v>
       </c>
@@ -7379,8 +7711,11 @@
       <c r="H6" s="3" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="7" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="I6" s="22" t="s">
+        <v>1059</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
         <v>161</v>
       </c>
@@ -7405,8 +7740,11 @@
       <c r="H7" s="5" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="8" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="I7" s="22" t="s">
+        <v>1059</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>167</v>
       </c>
@@ -7431,8 +7769,11 @@
       <c r="H8" s="3" t="s">
         <v>173</v>
       </c>
-    </row>
-    <row r="9" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="I8" s="22" t="s">
+        <v>1059</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
         <v>174</v>
       </c>
@@ -7457,8 +7798,11 @@
       <c r="H9" s="5" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="10" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="I9" s="22" t="s">
+        <v>1059</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>180</v>
       </c>
@@ -7483,8 +7827,11 @@
       <c r="H10" s="3" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="11" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="I10" s="24" t="s">
+        <v>1075</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
         <v>186</v>
       </c>
@@ -7508,6 +7855,9 @@
       </c>
       <c r="H11" s="5" t="s">
         <v>15</v>
+      </c>
+      <c r="I11" s="24" t="s">
+        <v>1075</v>
       </c>
     </row>
   </sheetData>
@@ -7518,19 +7868,21 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4FE07674-6098-4747-8826-848FDD58057F}">
-  <dimension ref="A1:H15"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:K15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.77734375" customWidth="1"/>
-    <col min="2" max="3" width="34.77734375" customWidth="1"/>
-    <col min="4" max="4" width="42.77734375" customWidth="1"/>
-    <col min="5" max="5" width="26.77734375" customWidth="1"/>
-    <col min="6" max="6" width="42.77734375" customWidth="1"/>
-    <col min="7" max="7" width="10.77734375" customWidth="1"/>
-    <col min="8" max="8" width="12.77734375" customWidth="1"/>
+    <col min="1" max="1" width="12.7109375" customWidth="1"/>
+    <col min="2" max="3" width="34.7109375" customWidth="1"/>
+    <col min="4" max="4" width="42.7109375" customWidth="1"/>
+    <col min="5" max="5" width="26.7109375" customWidth="1"/>
+    <col min="6" max="6" width="42.7109375" customWidth="1"/>
+    <col min="7" max="7" width="10.7109375" customWidth="1"/>
+    <col min="8" max="8" width="12.7109375" customWidth="1"/>
+    <col min="10" max="10" width="21.42578125" customWidth="1"/>
+    <col min="11" max="11" width="31.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -7555,8 +7907,17 @@
       <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="I1" s="16" t="s">
+        <v>1058</v>
+      </c>
+      <c r="J1" s="16" t="s">
+        <v>1071</v>
+      </c>
+      <c r="K1" s="16" t="s">
+        <v>1072</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>191</v>
       </c>
@@ -7581,8 +7942,11 @@
       <c r="H2" s="3" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="I2" s="25" t="s">
+        <v>1059</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>197</v>
       </c>
@@ -7607,8 +7971,14 @@
       <c r="H3" s="5" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="I3" s="25" t="s">
+        <v>1059</v>
+      </c>
+      <c r="J3" s="18" t="s">
+        <v>1076</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>203</v>
       </c>
@@ -7633,8 +8003,11 @@
       <c r="H4" s="3" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="I4" s="25" t="s">
+        <v>1059</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
         <v>209</v>
       </c>
@@ -7659,8 +8032,14 @@
       <c r="H5" s="5" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row r="6" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="I5" s="21" t="s">
+        <v>1067</v>
+      </c>
+      <c r="J5" s="18" t="s">
+        <v>1077</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>215</v>
       </c>
@@ -7685,8 +8064,14 @@
       <c r="H6" s="3" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="7" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="I6" s="21" t="s">
+        <v>1067</v>
+      </c>
+      <c r="J6" s="17" t="s">
+        <v>1078</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
         <v>221</v>
       </c>
@@ -7711,8 +8096,11 @@
       <c r="H7" s="5" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="8" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="I7" s="25" t="s">
+        <v>1059</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>227</v>
       </c>
@@ -7737,8 +8125,14 @@
       <c r="H8" s="3" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="9" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="I8" s="25" t="s">
+        <v>1059</v>
+      </c>
+      <c r="J8" s="18" t="s">
+        <v>1079</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" ht="75" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
         <v>232</v>
       </c>
@@ -7763,8 +8157,17 @@
       <c r="H9" s="5" t="s">
         <v>173</v>
       </c>
-    </row>
-    <row r="10" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="I9" s="25" t="s">
+        <v>1059</v>
+      </c>
+      <c r="J9" s="18" t="s">
+        <v>1080</v>
+      </c>
+      <c r="K9" s="18" t="s">
+        <v>1081</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>238</v>
       </c>
@@ -7789,8 +8192,11 @@
       <c r="H10" s="3" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row r="11" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="I10" s="25" t="s">
+        <v>1059</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
         <v>243</v>
       </c>
@@ -7815,8 +8221,11 @@
       <c r="H11" s="5" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row r="12" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="I11" s="25" t="s">
+        <v>1059</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>248</v>
       </c>
@@ -7841,8 +8250,11 @@
       <c r="H12" s="3" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row r="13" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="I12" s="25" t="s">
+        <v>1059</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
         <v>253</v>
       </c>
@@ -7867,8 +8279,11 @@
       <c r="H13" s="5" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="14" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="I13" s="25" t="s">
+        <v>1059</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>258</v>
       </c>
@@ -7893,8 +8308,11 @@
       <c r="H14" s="3" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="15" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="I14" s="25" t="s">
+        <v>1059</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
         <v>263</v>
       </c>
@@ -7918,6 +8336,9 @@
       </c>
       <c r="H15" s="5" t="s">
         <v>15</v>
+      </c>
+      <c r="I15" s="25" t="s">
+        <v>1059</v>
       </c>
     </row>
   </sheetData>
@@ -7928,19 +8349,22 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1501CF71-1BD9-48CE-A113-78E0494A13D4}">
-  <dimension ref="A1:H9"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:K9"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.77734375" customWidth="1"/>
-    <col min="2" max="3" width="34.77734375" customWidth="1"/>
-    <col min="4" max="4" width="42.77734375" customWidth="1"/>
-    <col min="5" max="5" width="26.77734375" customWidth="1"/>
-    <col min="6" max="6" width="42.77734375" customWidth="1"/>
-    <col min="7" max="7" width="10.77734375" customWidth="1"/>
-    <col min="8" max="8" width="12.77734375" customWidth="1"/>
+    <col min="1" max="1" width="12.7109375" customWidth="1"/>
+    <col min="2" max="3" width="34.7109375" customWidth="1"/>
+    <col min="4" max="4" width="42.7109375" customWidth="1"/>
+    <col min="5" max="5" width="26.7109375" customWidth="1"/>
+    <col min="6" max="6" width="42.7109375" customWidth="1"/>
+    <col min="7" max="7" width="10.7109375" customWidth="1"/>
+    <col min="8" max="8" width="12.7109375" customWidth="1"/>
+    <col min="9" max="9" width="11.7109375" customWidth="1"/>
+    <col min="10" max="10" width="38.42578125" customWidth="1"/>
+    <col min="11" max="11" width="38.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -7965,8 +8389,17 @@
       <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="I1" s="16" t="s">
+        <v>1058</v>
+      </c>
+      <c r="J1" s="16" t="s">
+        <v>1071</v>
+      </c>
+      <c r="K1" s="16" t="s">
+        <v>1072</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>268</v>
       </c>
@@ -7991,8 +8424,11 @@
       <c r="H2" s="3" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="I2" s="25" t="s">
+        <v>1059</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>274</v>
       </c>
@@ -8017,8 +8453,11 @@
       <c r="H3" s="5" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="I3" s="25" t="s">
+        <v>1059</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="37.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>280</v>
       </c>
@@ -8043,8 +8482,14 @@
       <c r="H4" s="3" t="s">
         <v>286</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="I4" s="21" t="s">
+        <v>1067</v>
+      </c>
+      <c r="J4" s="17" t="s">
+        <v>1082</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
         <v>287</v>
       </c>
@@ -8069,8 +8514,11 @@
       <c r="H5" s="5" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="6" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="I5" s="25" t="s">
+        <v>1059</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>293</v>
       </c>
@@ -8095,8 +8543,17 @@
       <c r="H6" s="3" t="s">
         <v>173</v>
       </c>
-    </row>
-    <row r="7" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="I6" s="25" t="s">
+        <v>1059</v>
+      </c>
+      <c r="J6" s="17" t="s">
+        <v>1083</v>
+      </c>
+      <c r="K6" s="17" t="s">
+        <v>1086</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
         <v>299</v>
       </c>
@@ -8121,8 +8578,14 @@
       <c r="H7" s="5" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="8" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="I7" s="25" t="s">
+        <v>1059</v>
+      </c>
+      <c r="J7" s="18" t="s">
+        <v>1084</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>305</v>
       </c>
@@ -8147,8 +8610,11 @@
       <c r="H8" s="3" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row r="9" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="I8" s="25" t="s">
+        <v>1059</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
         <v>311</v>
       </c>
@@ -8172,6 +8638,12 @@
       </c>
       <c r="H9" s="5" t="s">
         <v>286</v>
+      </c>
+      <c r="I9" s="21" t="s">
+        <v>1067</v>
+      </c>
+      <c r="J9" s="18" t="s">
+        <v>1085</v>
       </c>
     </row>
   </sheetData>
@@ -8182,19 +8654,22 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6D2FF9EC-FCAB-4361-B1BD-54388F7CC4AE}">
-  <dimension ref="A1:H13"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:K13"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.77734375" customWidth="1"/>
-    <col min="2" max="3" width="34.77734375" customWidth="1"/>
-    <col min="4" max="4" width="42.77734375" customWidth="1"/>
-    <col min="5" max="5" width="26.77734375" customWidth="1"/>
-    <col min="6" max="6" width="42.77734375" customWidth="1"/>
-    <col min="7" max="7" width="10.77734375" customWidth="1"/>
-    <col min="8" max="8" width="12.77734375" customWidth="1"/>
+    <col min="1" max="1" width="12.7109375" customWidth="1"/>
+    <col min="2" max="3" width="34.7109375" customWidth="1"/>
+    <col min="4" max="4" width="42.7109375" customWidth="1"/>
+    <col min="5" max="5" width="26.7109375" customWidth="1"/>
+    <col min="6" max="6" width="42.7109375" customWidth="1"/>
+    <col min="7" max="7" width="10.7109375" customWidth="1"/>
+    <col min="8" max="8" width="12.7109375" customWidth="1"/>
+    <col min="9" max="9" width="17" customWidth="1"/>
+    <col min="10" max="10" width="45.140625" customWidth="1"/>
+    <col min="11" max="11" width="33.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -8219,8 +8694,17 @@
       <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="I1" s="16" t="s">
+        <v>1058</v>
+      </c>
+      <c r="J1" s="16" t="s">
+        <v>1071</v>
+      </c>
+      <c r="K1" s="16" t="s">
+        <v>1072</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>317</v>
       </c>
@@ -8245,8 +8729,14 @@
       <c r="H2" s="3" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="I2" s="25" t="s">
+        <v>1059</v>
+      </c>
+      <c r="J2" s="17" t="s">
+        <v>1087</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>323</v>
       </c>
@@ -8271,8 +8761,14 @@
       <c r="H3" s="5" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="I3" s="21" t="s">
+        <v>1067</v>
+      </c>
+      <c r="J3" s="18" t="s">
+        <v>1088</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>328</v>
       </c>
@@ -8297,8 +8793,11 @@
       <c r="H4" s="3" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="I4" s="25" t="s">
+        <v>1059</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
         <v>334</v>
       </c>
@@ -8323,8 +8822,14 @@
       <c r="H5" s="5" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="6" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="I5" s="18" t="s">
+        <v>1089</v>
+      </c>
+      <c r="J5" s="18" t="s">
+        <v>1090</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>340</v>
       </c>
@@ -8349,8 +8854,11 @@
       <c r="H6" s="3" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="7" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="I6" s="25" t="s">
+        <v>1059</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
         <v>346</v>
       </c>
@@ -8375,8 +8883,14 @@
       <c r="H7" s="5" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="8" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="I7" s="21" t="s">
+        <v>1059</v>
+      </c>
+      <c r="J7" s="26" t="s">
+        <v>1091</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>352</v>
       </c>
@@ -8401,8 +8915,11 @@
       <c r="H8" s="3" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="9" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="I8" s="25" t="s">
+        <v>1059</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
         <v>358</v>
       </c>
@@ -8427,8 +8944,11 @@
       <c r="H9" s="5" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="10" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="I9" s="25" t="s">
+        <v>1059</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>364</v>
       </c>
@@ -8453,8 +8973,11 @@
       <c r="H10" s="3" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="11" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="I10" s="25" t="s">
+        <v>1059</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
         <v>370</v>
       </c>
@@ -8479,8 +9002,14 @@
       <c r="H11" s="5" t="s">
         <v>173</v>
       </c>
-    </row>
-    <row r="12" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="I11" s="25" t="s">
+        <v>1059</v>
+      </c>
+      <c r="J11" s="27" t="s">
+        <v>1092</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>376</v>
       </c>
@@ -8505,8 +9034,11 @@
       <c r="H12" s="3" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="13" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="I12" s="28" t="s">
+        <v>1062</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
         <v>382</v>
       </c>
@@ -8530,6 +9062,9 @@
       </c>
       <c r="H13" s="5" t="s">
         <v>286</v>
+      </c>
+      <c r="I13" s="28" t="s">
+        <v>1062</v>
       </c>
     </row>
   </sheetData>
@@ -8540,19 +9075,21 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B5671F5A-5323-441E-93DF-D3CC3173C937}">
-  <dimension ref="A1:H9"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:K9"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.77734375" customWidth="1"/>
-    <col min="2" max="3" width="34.77734375" customWidth="1"/>
-    <col min="4" max="4" width="42.77734375" customWidth="1"/>
-    <col min="5" max="5" width="26.77734375" customWidth="1"/>
-    <col min="6" max="6" width="42.77734375" customWidth="1"/>
-    <col min="7" max="7" width="10.77734375" customWidth="1"/>
-    <col min="8" max="8" width="12.77734375" customWidth="1"/>
+    <col min="1" max="1" width="12.7109375" customWidth="1"/>
+    <col min="2" max="3" width="34.7109375" customWidth="1"/>
+    <col min="4" max="4" width="42.7109375" customWidth="1"/>
+    <col min="5" max="5" width="26.7109375" customWidth="1"/>
+    <col min="6" max="6" width="42.7109375" customWidth="1"/>
+    <col min="7" max="7" width="10.7109375" customWidth="1"/>
+    <col min="8" max="8" width="12.7109375" customWidth="1"/>
+    <col min="9" max="9" width="25.140625" customWidth="1"/>
+    <col min="10" max="10" width="49" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -8577,8 +9114,17 @@
       <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="I1" s="16" t="s">
+        <v>1058</v>
+      </c>
+      <c r="J1" s="16" t="s">
+        <v>1071</v>
+      </c>
+      <c r="K1" s="16" t="s">
+        <v>1072</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>387</v>
       </c>
@@ -8603,8 +9149,11 @@
       <c r="H2" s="3" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="I2" s="25" t="s">
+        <v>1059</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>392</v>
       </c>
@@ -8629,8 +9178,17 @@
       <c r="H3" s="5" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="I3" s="21" t="s">
+        <v>1067</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>1093</v>
+      </c>
+      <c r="K3" t="s">
+        <v>1073</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>397</v>
       </c>
@@ -8655,8 +9213,11 @@
       <c r="H4" s="3" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="I4" s="25" t="s">
+        <v>1059</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
         <v>403</v>
       </c>
@@ -8681,8 +9242,11 @@
       <c r="H5" s="5" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="6" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="I5" s="25" t="s">
+        <v>1059</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>409</v>
       </c>
@@ -8707,8 +9271,11 @@
       <c r="H6" s="3" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="7" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="I6" s="25" t="s">
+        <v>1059</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
         <v>414</v>
       </c>
@@ -8733,8 +9300,11 @@
       <c r="H7" s="5" t="s">
         <v>173</v>
       </c>
-    </row>
-    <row r="8" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="I7" s="25" t="s">
+        <v>1059</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>420</v>
       </c>
@@ -8759,8 +9329,11 @@
       <c r="H8" s="3" t="s">
         <v>286</v>
       </c>
-    </row>
-    <row r="9" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="I8" s="25" t="s">
+        <v>1059</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
         <v>426</v>
       </c>
@@ -8784,29 +9357,35 @@
       </c>
       <c r="H9" s="5" t="s">
         <v>15</v>
+      </c>
+      <c r="I9" s="25" t="s">
+        <v>1059</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:H9" xr:uid="{B5671F5A-5323-441E-93DF-D3CC3173C937}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0DFB3D39-1786-40A1-9AE4-F60CE24805AD}">
-  <dimension ref="A1:H9"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:K9"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.77734375" customWidth="1"/>
-    <col min="2" max="3" width="34.77734375" customWidth="1"/>
-    <col min="4" max="4" width="42.77734375" customWidth="1"/>
-    <col min="5" max="5" width="26.77734375" customWidth="1"/>
-    <col min="6" max="6" width="42.77734375" customWidth="1"/>
-    <col min="7" max="7" width="10.77734375" customWidth="1"/>
-    <col min="8" max="8" width="12.77734375" customWidth="1"/>
+    <col min="1" max="1" width="12.7109375" customWidth="1"/>
+    <col min="2" max="3" width="34.7109375" customWidth="1"/>
+    <col min="4" max="4" width="42.7109375" customWidth="1"/>
+    <col min="5" max="5" width="26.7109375" customWidth="1"/>
+    <col min="6" max="6" width="42.7109375" customWidth="1"/>
+    <col min="7" max="7" width="10.7109375" customWidth="1"/>
+    <col min="8" max="8" width="12.7109375" customWidth="1"/>
+    <col min="10" max="10" width="14.7109375" customWidth="1"/>
+    <col min="11" max="11" width="40.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -8831,8 +9410,17 @@
       <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="I1" s="16" t="s">
+        <v>1058</v>
+      </c>
+      <c r="J1" s="16" t="s">
+        <v>1071</v>
+      </c>
+      <c r="K1" s="16" t="s">
+        <v>1072</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>432</v>
       </c>
@@ -8858,7 +9446,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>437</v>
       </c>
@@ -8884,7 +9472,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>443</v>
       </c>
@@ -8910,7 +9498,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
         <v>448</v>
       </c>
@@ -8936,7 +9524,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>453</v>
       </c>
@@ -8962,7 +9550,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
         <v>459</v>
       </c>
@@ -8988,7 +9576,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>465</v>
       </c>
@@ -9014,7 +9602,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
         <v>471</v>
       </c>
@@ -9049,18 +9637,18 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EFCBC1D3-621F-4260-9467-218A26FDEB8F}">
   <dimension ref="A1:H7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.77734375" customWidth="1"/>
-    <col min="2" max="3" width="34.77734375" customWidth="1"/>
-    <col min="4" max="4" width="42.77734375" customWidth="1"/>
-    <col min="5" max="5" width="26.77734375" customWidth="1"/>
-    <col min="6" max="6" width="42.77734375" customWidth="1"/>
-    <col min="7" max="7" width="10.77734375" customWidth="1"/>
-    <col min="8" max="8" width="12.77734375" customWidth="1"/>
+    <col min="1" max="1" width="12.7109375" customWidth="1"/>
+    <col min="2" max="3" width="34.7109375" customWidth="1"/>
+    <col min="4" max="4" width="42.7109375" customWidth="1"/>
+    <col min="5" max="5" width="26.7109375" customWidth="1"/>
+    <col min="6" max="6" width="42.7109375" customWidth="1"/>
+    <col min="7" max="7" width="10.7109375" customWidth="1"/>
+    <col min="8" max="8" width="12.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -9086,7 +9674,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>477</v>
       </c>
@@ -9112,7 +9700,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>482</v>
       </c>
@@ -9138,7 +9726,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>487</v>
       </c>
@@ -9164,7 +9752,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
         <v>492</v>
       </c>
@@ -9190,7 +9778,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>498</v>
       </c>
@@ -9216,7 +9804,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
         <v>504</v>
       </c>

</xml_diff>

<commit_message>
* Making RunTime settings order by!
</commit_message>
<xml_diff>
--- a/docs/SFTPManager-Test-Plan.xlsx
+++ b/docs/SFTPManager-Test-Plan.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\joema\Downloads\sftp-manager\sftp-manager\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18D87BE3-8117-47E1-B9AE-00657FA00DE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71AB6B6C-E3DA-408D-AEDF-A8D2313A7AD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="27885" windowHeight="16440" firstSheet="5" activeTab="7" xr2:uid="{3AB46E1C-6979-4AE0-A30D-F087EBE6ECB8}"/>
+    <workbookView xWindow="30165" yWindow="2100" windowWidth="20730" windowHeight="11835" firstSheet="5" activeTab="8" xr2:uid="{3AB46E1C-6979-4AE0-A30D-F087EBE6ECB8}"/>
   </bookViews>
   <sheets>
     <sheet name="Index" sheetId="1" r:id="rId1"/>
@@ -71,7 +71,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1688" uniqueCount="1094">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1711" uniqueCount="1102">
   <si>
     <t>ID</t>
   </si>
@@ -3353,6 +3353,30 @@
   </si>
   <si>
     <t>2026-07-31 07:10:01,067 mod_wrap2/2.0.7[436052]: warning: bad net/mask expression: '172.105.168.0/24'. Individual IPS work</t>
+  </si>
+  <si>
+    <t>When I set BASIC plan to 0.00 and set Paid_to_date to the current date, it refused to bill.</t>
+  </si>
+  <si>
+    <t>We only ever have ONE trial plan.</t>
+  </si>
+  <si>
+    <t>Changed BASIC plan to have blank storage.</t>
+  </si>
+  <si>
+    <t>It isn't deleted. There are no errors.</t>
+  </si>
+  <si>
+    <t>trial option not shown.</t>
+  </si>
+  <si>
+    <t>Says Save Failed. Good</t>
+  </si>
+  <si>
+    <t>SKIPPING</t>
+  </si>
+  <si>
+    <t>Not going to delete</t>
   </si>
 </sst>
 </file>
@@ -3539,7 +3563,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -3607,6 +3631,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -9381,7 +9408,7 @@
     <col min="6" max="6" width="42.7109375" customWidth="1"/>
     <col min="7" max="7" width="10.7109375" customWidth="1"/>
     <col min="8" max="8" width="12.7109375" customWidth="1"/>
-    <col min="10" max="10" width="14.7109375" customWidth="1"/>
+    <col min="10" max="10" width="50.28515625" customWidth="1"/>
     <col min="11" max="11" width="40.85546875" customWidth="1"/>
   </cols>
   <sheetData>
@@ -9445,6 +9472,12 @@
       <c r="H2" s="3" t="s">
         <v>15</v>
       </c>
+      <c r="I2" s="25" t="s">
+        <v>1059</v>
+      </c>
+      <c r="J2" s="17" t="s">
+        <v>1094</v>
+      </c>
     </row>
     <row r="3" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
@@ -9471,6 +9504,12 @@
       <c r="H3" s="5" t="s">
         <v>15</v>
       </c>
+      <c r="I3" s="29" t="s">
+        <v>1089</v>
+      </c>
+      <c r="J3" s="29" t="s">
+        <v>1095</v>
+      </c>
     </row>
     <row r="4" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
@@ -9497,6 +9536,12 @@
       <c r="H4" s="3" t="s">
         <v>15</v>
       </c>
+      <c r="I4" s="25" t="s">
+        <v>1059</v>
+      </c>
+      <c r="J4" s="17" t="s">
+        <v>1096</v>
+      </c>
     </row>
     <row r="5" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
@@ -9523,6 +9568,7 @@
       <c r="H5" s="5" t="s">
         <v>22</v>
       </c>
+      <c r="I5" s="17"/>
     </row>
     <row r="6" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
@@ -9549,6 +9595,9 @@
       <c r="H6" s="3" t="s">
         <v>286</v>
       </c>
+      <c r="I6" s="25" t="s">
+        <v>1059</v>
+      </c>
     </row>
     <row r="7" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
@@ -9575,6 +9624,9 @@
       <c r="H7" s="5" t="s">
         <v>131</v>
       </c>
+      <c r="I7" s="25" t="s">
+        <v>1059</v>
+      </c>
     </row>
     <row r="8" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
@@ -9601,6 +9653,12 @@
       <c r="H8" s="3" t="s">
         <v>286</v>
       </c>
+      <c r="I8" s="25" t="s">
+        <v>1059</v>
+      </c>
+      <c r="J8" s="17" t="s">
+        <v>1097</v>
+      </c>
     </row>
     <row r="9" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
@@ -9626,6 +9684,9 @@
       </c>
       <c r="H9" s="5" t="s">
         <v>131</v>
+      </c>
+      <c r="I9" s="25" t="s">
+        <v>1059</v>
       </c>
     </row>
   </sheetData>
@@ -9636,7 +9697,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EFCBC1D3-621F-4260-9467-218A26FDEB8F}">
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:K7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
@@ -9646,9 +9707,10 @@
     <col min="6" max="6" width="42.7109375" customWidth="1"/>
     <col min="7" max="7" width="10.7109375" customWidth="1"/>
     <col min="8" max="8" width="12.7109375" customWidth="1"/>
+    <col min="10" max="10" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -9673,8 +9735,17 @@
       <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="I1" s="16" t="s">
+        <v>1058</v>
+      </c>
+      <c r="J1" s="16" t="s">
+        <v>1071</v>
+      </c>
+      <c r="K1" s="16" t="s">
+        <v>1072</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>477</v>
       </c>
@@ -9699,8 +9770,11 @@
       <c r="H2" s="3" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" ht="60" x14ac:dyDescent="0.25">
+      <c r="I2" s="25" t="s">
+        <v>1059</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>482</v>
       </c>
@@ -9725,8 +9799,14 @@
       <c r="H3" s="5" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="I3" s="25" t="s">
+        <v>1059</v>
+      </c>
+      <c r="J3" s="29" t="s">
+        <v>1098</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>487</v>
       </c>
@@ -9751,8 +9831,11 @@
       <c r="H4" s="3" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="I4" s="25" t="s">
+        <v>1059</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
         <v>492</v>
       </c>
@@ -9777,8 +9860,14 @@
       <c r="H5" s="5" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="6" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="I5" s="25" t="s">
+        <v>1059</v>
+      </c>
+      <c r="J5" s="29" t="s">
+        <v>1099</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>498</v>
       </c>
@@ -9803,8 +9892,14 @@
       <c r="H6" s="3" t="s">
         <v>286</v>
       </c>
-    </row>
-    <row r="7" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="I6" s="25" t="s">
+        <v>1100</v>
+      </c>
+      <c r="J6" s="17" t="s">
+        <v>1101</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
         <v>504</v>
       </c>
@@ -9828,6 +9923,9 @@
       </c>
       <c r="H7" s="5" t="s">
         <v>15</v>
+      </c>
+      <c r="I7" s="25" t="s">
+        <v>1059</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
* Updated to 14 day trial period. (From 7)
</commit_message>
<xml_diff>
--- a/docs/SFTPManager-Test-Plan.xlsx
+++ b/docs/SFTPManager-Test-Plan.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\joema\Downloads\sftp-manager\sftp-manager\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71AB6B6C-E3DA-408D-AEDF-A8D2313A7AD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68373DCF-1AD2-40B7-A1D5-3558E57531F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30165" yWindow="2100" windowWidth="20730" windowHeight="11835" firstSheet="5" activeTab="8" xr2:uid="{3AB46E1C-6979-4AE0-A30D-F087EBE6ECB8}"/>
+    <workbookView xWindow="30630" yWindow="2175" windowWidth="25845" windowHeight="11835" firstSheet="8" activeTab="9" xr2:uid="{3AB46E1C-6979-4AE0-A30D-F087EBE6ECB8}"/>
   </bookViews>
   <sheets>
     <sheet name="Index" sheetId="1" r:id="rId1"/>
@@ -71,7 +71,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1711" uniqueCount="1102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1714" uniqueCount="1102">
   <si>
     <t>ID</t>
   </si>
@@ -4206,7 +4206,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE4B2888-C380-42AB-B6FF-7902ECD4725D}">
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:K16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
@@ -4216,9 +4216,11 @@
     <col min="6" max="6" width="42.7109375" customWidth="1"/>
     <col min="7" max="7" width="10.7109375" customWidth="1"/>
     <col min="8" max="8" width="12.7109375" customWidth="1"/>
+    <col min="9" max="9" width="17" customWidth="1"/>
+    <col min="11" max="11" width="17.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -4243,8 +4245,17 @@
       <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="I1" s="16" t="s">
+        <v>1058</v>
+      </c>
+      <c r="J1" s="16" t="s">
+        <v>1071</v>
+      </c>
+      <c r="K1" s="16" t="s">
+        <v>1072</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>509</v>
       </c>
@@ -4270,7 +4281,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>515</v>
       </c>
@@ -4296,7 +4307,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>521</v>
       </c>
@@ -4322,7 +4333,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
         <v>527</v>
       </c>
@@ -4348,7 +4359,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>532</v>
       </c>
@@ -4374,7 +4385,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
         <v>538</v>
       </c>
@@ -4400,7 +4411,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="60" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>544</v>
       </c>
@@ -4426,7 +4437,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
         <v>550</v>
       </c>
@@ -4452,7 +4463,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>555</v>
       </c>
@@ -4478,7 +4489,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="60" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
         <v>560</v>
       </c>
@@ -4504,7 +4515,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>566</v>
       </c>
@@ -4530,7 +4541,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
         <v>572</v>
       </c>
@@ -4556,7 +4567,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>578</v>
       </c>
@@ -4582,7 +4593,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
         <v>583</v>
       </c>
@@ -4608,7 +4619,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>589</v>
       </c>

</xml_diff>